<commit_message>
Update logbook from 20251126
</commit_message>
<xml_diff>
--- a/data/VMP/20251126/Level0/Logbook_Zug_20251126.xlsx
+++ b/data/VMP/20251126/Level0/Logbook_Zug_20251126.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unils-my.sharepoint.com/personal/tomy_doda_unil_ch/Documents/Projects-GSE42572/3-Zug/turbulence-lakezug/data/VMP/20251126/Level0/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="309" documentId="13_ncr:1_{F97EAE30-667A-4A71-BFDC-08A402DAEF65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{919A781C-1B60-4C4B-BF84-28BA2A55BC29}"/>
+  <xr:revisionPtr revIDLastSave="317" documentId="13_ncr:1_{F97EAE30-667A-4A71-BFDC-08A402DAEF65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{09C6FDD0-EF5E-4378-BEF6-0BB430E15C87}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Logbook_Zug" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="43">
   <si>
     <t>Date</t>
   </si>
@@ -131,9 +131,6 @@
     <t>VMP003</t>
   </si>
   <si>
-    <t>PSB01</t>
-  </si>
-  <si>
     <t>VMP004</t>
   </si>
   <si>
@@ -146,24 +143,12 @@
     <t>VMP010</t>
   </si>
   <si>
-    <t>PSB02</t>
-  </si>
-  <si>
     <t>No fluoro (cap on), vibrations at 120 m, stop winch at 170m, winch up at 185 m, VMP goes up at 190m</t>
   </si>
   <si>
     <t xml:space="preserve">No fluoro (cap on), vibrations over the top 15 m </t>
   </si>
   <si>
-    <t>PC01</t>
-  </si>
-  <si>
-    <t>PC02</t>
-  </si>
-  <si>
-    <t>PC03</t>
-  </si>
-  <si>
     <t>Windy, vibrations over the top 25 m</t>
   </si>
   <si>
@@ -174,6 +159,12 @@
   </si>
   <si>
     <t>P_offset_dbar</t>
+  </si>
+  <si>
+    <t>PS</t>
+  </si>
+  <si>
+    <t>PC</t>
   </si>
 </sst>
 </file>
@@ -890,7 +881,7 @@
         <v>26</v>
       </c>
       <c r="Y1" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="Z1" s="7" t="s">
         <v>1</v>
@@ -1011,7 +1002,7 @@
         <v>216834</v>
       </c>
       <c r="O3" s="35" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="P3" s="35">
         <v>200</v>
@@ -1038,12 +1029,12 @@
         <v>-0.15</v>
       </c>
       <c r="Z3" s="41" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:27" s="15" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B4" s="12">
         <v>2</v>
@@ -1077,7 +1068,7 @@
         <v>216813</v>
       </c>
       <c r="O4" s="12" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="P4" s="12">
         <v>200</v>
@@ -1104,13 +1095,13 @@
         <v>-0.15</v>
       </c>
       <c r="Z4" s="42" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="AA4"/>
     </row>
     <row r="5" spans="1:27" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="19" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B5" s="19">
         <v>3</v>
@@ -1144,7 +1135,7 @@
         <v>218781</v>
       </c>
       <c r="O5" s="19" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="P5" s="19">
         <v>170</v>
@@ -1171,13 +1162,13 @@
         <v>-0.15</v>
       </c>
       <c r="Z5" s="43" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="AA5"/>
     </row>
     <row r="6" spans="1:27" s="17" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="22" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B6" s="22">
         <v>4</v>
@@ -1211,7 +1202,7 @@
         <v>218711</v>
       </c>
       <c r="O6" s="22" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="P6" s="22">
         <v>170</v>
@@ -1238,13 +1229,13 @@
         <v>-0.15</v>
       </c>
       <c r="Z6" s="44" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AA6"/>
     </row>
     <row r="7" spans="1:27" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="25" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B7" s="25">
         <v>5</v>
@@ -1278,7 +1269,7 @@
         <v>218702</v>
       </c>
       <c r="O7" s="25" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="P7" s="25">
         <v>170</v>
@@ -1305,7 +1296,7 @@
         <v>-0.15</v>
       </c>
       <c r="Z7" s="45" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="AA7"/>
     </row>

</xml_diff>

<commit_message>
Update logbook 20251126: use same profile names as for CTD
</commit_message>
<xml_diff>
--- a/data/VMP/20251126/Level0/Logbook_Zug_20251126.xlsx
+++ b/data/VMP/20251126/Level0/Logbook_Zug_20251126.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unils-my.sharepoint.com/personal/tomy_doda_unil_ch/Documents/Projects-GSE42572/3-Zug/turbulence-lakezug/data/VMP/20251126/Level0/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="317" documentId="13_ncr:1_{F97EAE30-667A-4A71-BFDC-08A402DAEF65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{09C6FDD0-EF5E-4378-BEF6-0BB430E15C87}"/>
+  <xr:revisionPtr revIDLastSave="322" documentId="13_ncr:1_{F97EAE30-667A-4A71-BFDC-08A402DAEF65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B1979BB8-D183-42F8-96FB-3DCDB9B89D59}"/>
   <bookViews>
-    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Logbook_Zug" sheetId="1" r:id="rId1"/>
@@ -161,10 +161,10 @@
     <t>P_offset_dbar</t>
   </si>
   <si>
-    <t>PS</t>
-  </si>
-  <si>
-    <t>PC</t>
+    <t>VMPS</t>
+  </si>
+  <si>
+    <t>VMPC</t>
   </si>
 </sst>
 </file>

</xml_diff>